<commit_message>
ASP-5596 Add Assay and Consumable filter information to report header
</commit_message>
<xml_diff>
--- a/api/templates/pk_missing_cartridges_report/en.xlsx
+++ b/api/templates/pk_missing_cartridges_report/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\opewix\dev\sysone\sources\aspect\api\templates\pk_missing_cartridges_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05E2C92F-73D6-4C85-8AB3-0B416EB36E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39702524-C3BA-454A-BF59-21A866673F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11505" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Missing Lots" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t>&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t>Assays: &lt;Assays&gt;</t>
+  </si>
+  <si>
+    <t>Consumables: &lt;Consumables&gt;</t>
   </si>
 </sst>
 </file>
@@ -664,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5" style="2" customWidth="1"/>
@@ -709,63 +715,77 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+    <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B9" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="10" spans="1:7" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
ASP-5596 Remove min date, rename column and add orderby to query
</commit_message>
<xml_diff>
--- a/api/templates/pk_missing_cartridges_report/en.xlsx
+++ b/api/templates/pk_missing_cartridges_report/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\opewix\dev\sysone\sources\aspect\api\templates\pk_missing_cartridges_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39702524-C3BA-454A-BF59-21A866673F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E0BA2C-55CC-4010-974B-8B43C88F8442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,18 +30,12 @@
     <t>&lt;Table&gt;</t>
   </si>
   <si>
-    <t>&lt;endedOn&gt;</t>
-  </si>
-  <si>
     <t>Site</t>
   </si>
   <si>
     <t>Printed on &lt;Dates&gt;</t>
   </si>
   <si>
-    <t>Ended On</t>
-  </si>
-  <si>
     <t>Province</t>
   </si>
   <si>
@@ -91,6 +85,12 @@
   </si>
   <si>
     <t>Consumables: &lt;Consumables&gt;</t>
+  </si>
+  <si>
+    <t>Test Ended On</t>
+  </si>
+  <si>
+    <t>&lt;testEndedOn&gt;</t>
   </si>
 </sst>
 </file>
@@ -684,47 +684,47 @@
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
@@ -736,48 +736,48 @@
     </row>
     <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="F9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>7</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>13</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Changed orther of missing lots report columns
</commit_message>
<xml_diff>
--- a/api/templates/pk_missing_cartridges_report/en.xlsx
+++ b/api/templates/pk_missing_cartridges_report/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26327"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\pk_missing_cartridges_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\pk_missing_cartridges_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80F015B-11D2-4719-BA13-1A6E1A3E4391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15996" tabRatio="815"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Missing Lots" sheetId="1" r:id="rId1"/>
@@ -92,16 +93,16 @@
     <t>&lt;testEndedOn&gt;</t>
   </si>
   <si>
-    <t>Consumables</t>
-  </si>
-  <si>
     <t>&lt;consumableName&gt;</t>
+  </si>
+  <si>
+    <t>Consumable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -337,7 +338,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -674,7 +675,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H12"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -685,7 +686,7 @@
     <col min="5" max="5" width="28.59765625" style="1" customWidth="1"/>
     <col min="6" max="6" width="21.3984375" style="1" customWidth="1"/>
     <col min="7" max="7" width="21.19921875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.59765625" customWidth="1"/>
+    <col min="8" max="8" width="34.69921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.4">
@@ -754,16 +755,16 @@
         <v>4</v>
       </c>
       <c r="E9" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="10" t="s">
         <v>7</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="1" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -780,16 +781,16 @@
         <v>8</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>13</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>